<commit_message>
docs: deepen Hynix peer, vintage and company analysis framework
</commit_message>
<xml_diff>
--- a/model/SK_hynix_equity_research_final.xlsx
+++ b/model/SK_hynix_equity_research_final.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra29c69387c4049c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="R0ec31433932d4388"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R976f1ec42f6c4ca6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HBM Build" sheetId="4" r:id="R9cffd69de9d24e76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="5" r:id="R4532c97a66434eba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" r:id="R66dc3a130f534068"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="7" r:id="R102b915c04cb41f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="8" r:id="R99e037692a9b47aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="9" r:id="Rde11aa04349b4d87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R33c7b8cdcd2649a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="R2fd1dbaf8dab4638"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R28c35e5ef98c48a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HBM Build" sheetId="4" r:id="R066de7dfa4374f82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="5" r:id="R7c7762131c7e451c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" r:id="R1bc263dd514d47e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="7" r:id="Rb191f6435fc143d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="8" r:id="R536b6e46bb6b434d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="9" r:id="Rc50fd0b0ffc245af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -27,7 +27,7 @@
     <x:numFmt numFmtId="202" formatCode="#,##0.0"/>
     <x:numFmt numFmtId="203" formatCode="0.0x"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -71,8 +71,19 @@
       <x:color rgb="FF1F2937"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF333333"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -114,8 +125,38 @@
         <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="10">
     <x:border>
       <x:left/>
       <x:right/>
@@ -138,11 +179,91 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:right>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFC8D2DC"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="91">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -223,6 +344,97 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -726,14 +938,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="26" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="26" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1174,6 +1386,226 @@
       </x:c>
       <x:c r="B25" s="35" t="str">
         <x:v>https://stockanalysis.com/quote/krx/000660/history/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="82" t="str">
+        <x:v>Valuation vintage controls</x:v>
+      </x:c>
+      <x:c r="B27" s="82"/>
+      <x:c r="C27" s="82"/>
+      <x:c r="D27" s="82"/>
+      <x:c r="E27" s="82"/>
+      <x:c r="F27" s="82"/>
+      <x:c r="G27" s="82"/>
+      <x:c r="H27" s="82"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="85" t="str">
+        <x:v>Control</x:v>
+      </x:c>
+      <x:c r="B28" s="86" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C28" s="86" t="str">
+        <x:v>Definition</x:v>
+      </x:c>
+      <x:c r="D28" s="86" t="str">
+        <x:v>Source / owner</x:v>
+      </x:c>
+      <x:c r="E28" s="86" t="str">
+        <x:v>Data status</x:v>
+      </x:c>
+      <x:c r="F28" s="86" t="str">
+        <x:v>Refresh event</x:v>
+      </x:c>
+      <x:c r="G28" s="86" t="str">
+        <x:v>Model use</x:v>
+      </x:c>
+      <x:c r="H28" s="87" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="61" t="str">
+        <x:v>Valuation as-of</x:v>
+      </x:c>
+      <x:c r="B29" s="57" t="str">
+        <x:v>2026-10-07</x:v>
+      </x:c>
+      <x:c r="C29" s="57" t="str">
+        <x:v>KRX closing price date</x:v>
+      </x:c>
+      <x:c r="D29" s="57" t="str">
+        <x:v>KRX / market data</x:v>
+      </x:c>
+      <x:c r="E29" s="57" t="str">
+        <x:v>Model vintage</x:v>
+      </x:c>
+      <x:c r="F29" s="57" t="str">
+        <x:v>Every valuation refresh</x:v>
+      </x:c>
+      <x:c r="G29" s="57" t="str">
+        <x:v>Summary, DCF, PER</x:v>
+      </x:c>
+      <x:c r="H29" s="62" t="str">
+        <x:v>Use a trading day</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="24" hidden="0" customHeight="1">
+      <x:c r="A30" s="61" t="str">
+        <x:v>Information cutoff</x:v>
+      </x:c>
+      <x:c r="B30" s="57" t="str">
+        <x:v>2026-10-07 close</x:v>
+      </x:c>
+      <x:c r="C30" s="57" t="str">
+        <x:v>Information public by this cutoff</x:v>
+      </x:c>
+      <x:c r="D30" s="57" t="str">
+        <x:v>DART and company IR</x:v>
+      </x:c>
+      <x:c r="E30" s="57" t="str">
+        <x:v>Model vintage</x:v>
+      </x:c>
+      <x:c r="F30" s="57" t="str">
+        <x:v>Every new disclosure</x:v>
+      </x:c>
+      <x:c r="G30" s="57" t="str">
+        <x:v>All actuals and forecast inputs</x:v>
+      </x:c>
+      <x:c r="H30" s="62" t="str">
+        <x:v>After-close releases roll to next trading-day vintage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="61" t="str">
+        <x:v>Latest annual actual</x:v>
+      </x:c>
+      <x:c r="B31" s="57" t="str">
+        <x:v>FY2025</x:v>
+      </x:c>
+      <x:c r="C31" s="57" t="str">
+        <x:v>Latest annual period in current model</x:v>
+      </x:c>
+      <x:c r="D31" s="57" t="str">
+        <x:v>SK hynix FY25 results</x:v>
+      </x:c>
+      <x:c r="E31" s="57" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F31" s="57" t="str">
+        <x:v>Annual filing</x:v>
+      </x:c>
+      <x:c r="G31" s="57" t="str">
+        <x:v>Actuals, Forecast, SOTP, RIM</x:v>
+      </x:c>
+      <x:c r="H31" s="62" t="str">
+        <x:v>Keep audited/annual period label</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="24" hidden="0" customHeight="1">
+      <x:c r="A32" s="61" t="str">
+        <x:v>Latest quarterly actual</x:v>
+      </x:c>
+      <x:c r="B32" s="57" t="str">
+        <x:v>2Q2026</x:v>
+      </x:c>
+      <x:c r="C32" s="57" t="str">
+        <x:v>Latest quarter in current model</x:v>
+      </x:c>
+      <x:c r="D32" s="57" t="str">
+        <x:v>SK hynix 2Q26 results</x:v>
+      </x:c>
+      <x:c r="E32" s="57" t="str">
+        <x:v>Preliminary company release</x:v>
+      </x:c>
+      <x:c r="F32" s="57" t="str">
+        <x:v>Quarterly release / filing</x:v>
+      </x:c>
+      <x:c r="G32" s="57" t="str">
+        <x:v>Actuals, Forecast, HBM Build</x:v>
+      </x:c>
+      <x:c r="H32" s="62" t="str">
+        <x:v>Do not confuse quarter and half-year cumulative values</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="24" hidden="0" customHeight="1">
+      <x:c r="A33" s="61" t="str">
+        <x:v>Forecast vintage</x:v>
+      </x:c>
+      <x:c r="B33" s="57" t="str">
+        <x:v>2026-10-07 analyst case</x:v>
+      </x:c>
+      <x:c r="C33" s="57" t="str">
+        <x:v>Analyst base/bull/bear assumptions as of cutoff</x:v>
+      </x:c>
+      <x:c r="D33" s="57" t="str">
+        <x:v>Analyst model</x:v>
+      </x:c>
+      <x:c r="E33" s="57" t="str">
+        <x:v>Estimate</x:v>
+      </x:c>
+      <x:c r="F33" s="57" t="str">
+        <x:v>Each earnings / outlook revision</x:v>
+      </x:c>
+      <x:c r="G33" s="57" t="str">
+        <x:v>Forecast and all valuation tabs</x:v>
+      </x:c>
+      <x:c r="H33" s="62" t="str">
+        <x:v>Not a company guidance or consensus snapshot</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="24" hidden="0" customHeight="1">
+      <x:c r="A34" s="61" t="str">
+        <x:v>Market price date</x:v>
+      </x:c>
+      <x:c r="B34" s="57" t="str">
+        <x:v>2026-10-07</x:v>
+      </x:c>
+      <x:c r="C34" s="57" t="str">
+        <x:v>Closing price; KRW/share</x:v>
+      </x:c>
+      <x:c r="D34" s="57" t="str">
+        <x:v>StockAnalysis KRX 000660 history</x:v>
+      </x:c>
+      <x:c r="E34" s="57" t="str">
+        <x:v>Market input</x:v>
+      </x:c>
+      <x:c r="F34" s="57" t="str">
+        <x:v>Every valuation refresh</x:v>
+      </x:c>
+      <x:c r="G34" s="57" t="str">
+        <x:v>Summary, PER</x:v>
+      </x:c>
+      <x:c r="H34" s="62" t="str">
+        <x:v>Verify against exchange data before refresh</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="24" hidden="0" customHeight="1">
+      <x:c r="A35" s="70" t="str">
+        <x:v>Diluted shares date</x:v>
+      </x:c>
+      <x:c r="B35" s="71" t="str">
+        <x:v>2026-10-07 assumption</x:v>
+      </x:c>
+      <x:c r="C35" s="71" t="str">
+        <x:v>700 million forecast shares in current model</x:v>
+      </x:c>
+      <x:c r="D35" s="71" t="str">
+        <x:v>Analyst input; source reconciliation required</x:v>
+      </x:c>
+      <x:c r="E35" s="71" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="F35" s="71" t="str">
+        <x:v>Corporate action / issuance</x:v>
+      </x:c>
+      <x:c r="G35" s="71" t="str">
+        <x:v>Per-share values</x:v>
+      </x:c>
+      <x:c r="H35" s="72" t="str">
+        <x:v>Do not label as reported actual shares</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2936,12 +3368,12 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="46" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
   </x:cols>
@@ -2960,7 +3392,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Micron is the only direct PER anchor. Other companies are used only at segment or qualitative level.</x:v>
+        <x:v>Micron is the sole direct economics anchor. PER bridge values are analyst scenario inputs until historical calibration; see rows 30–45.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -3336,6 +3768,294 @@
       <x:c r="B27" s="40" t="n">
         <x:f>B26*E22</x:f>
         <x:v>1828571.428571429</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="82" t="str">
+        <x:v>Peer eligibility and multiple calibration</x:v>
+      </x:c>
+      <x:c r="B30" s="82"/>
+      <x:c r="C30" s="82"/>
+      <x:c r="D30" s="82"/>
+      <x:c r="E30" s="82"/>
+      <x:c r="F30" s="82"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="85" t="str">
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="B31" s="86" t="str">
+        <x:v>Minimum evidence</x:v>
+      </x:c>
+      <x:c r="C31" s="86" t="str">
+        <x:v>Micron</x:v>
+      </x:c>
+      <x:c r="D31" s="86" t="str">
+        <x:v>Samsung memory</x:v>
+      </x:c>
+      <x:c r="E31" s="86" t="str">
+        <x:v>NAND peers</x:v>
+      </x:c>
+      <x:c r="F31" s="87" t="str">
+        <x:v>If test fails</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="36" hidden="0" customHeight="1">
+      <x:c r="A32" s="61" t="str">
+        <x:v>Earnings source</x:v>
+      </x:c>
+      <x:c r="B32" s="57" t="str">
+        <x:v>Own memory manufacturing is a central profit source; reported and segment data can be reconciled</x:v>
+      </x:c>
+      <x:c r="C32" s="57" t="str">
+        <x:v>Direct anchor candidate</x:v>
+      </x:c>
+      <x:c r="D32" s="57" t="str">
+        <x:v>Segment operations only</x:v>
+      </x:c>
+      <x:c r="E32" s="57" t="str">
+        <x:v>NAND segment only</x:v>
+      </x:c>
+      <x:c r="F32" s="62" t="str">
+        <x:v>Move to operating or product-demand reference</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="24" hidden="0" customHeight="1">
+      <x:c r="A33" s="61" t="str">
+        <x:v>Price cycle</x:v>
+      </x:c>
+      <x:c r="B33" s="57" t="str">
+        <x:v>DRAM/NAND pricing, bit supply and inventory visibly affect earnings</x:v>
+      </x:c>
+      <x:c r="C33" s="57" t="str">
+        <x:v>Direct anchor candidate</x:v>
+      </x:c>
+      <x:c r="D33" s="57" t="str">
+        <x:v>Memory segment only</x:v>
+      </x:c>
+      <x:c r="E33" s="57" t="str">
+        <x:v>NAND cycle only</x:v>
+      </x:c>
+      <x:c r="F33" s="62" t="str">
+        <x:v>Do not combine with DRAM/HBM earnings multiple</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="24" hidden="0" customHeight="1">
+      <x:c r="A34" s="61" t="str">
+        <x:v>Capital intensity</x:v>
+      </x:c>
+      <x:c r="B34" s="57" t="str">
+        <x:v>Own fabs, depreciation, inventory and material CAPEX are in the economics</x:v>
+      </x:c>
+      <x:c r="C34" s="57" t="str">
+        <x:v>Direct anchor candidate</x:v>
+      </x:c>
+      <x:c r="D34" s="57" t="str">
+        <x:v>Segment CAPEX if disclosed</x:v>
+      </x:c>
+      <x:c r="E34" s="57" t="str">
+        <x:v>NAND investment only</x:v>
+      </x:c>
+      <x:c r="F34" s="62" t="str">
+        <x:v>Use for operating checks, not direct PER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="24" hidden="0" customHeight="1">
+      <x:c r="A35" s="61" t="str">
+        <x:v>Earnings normalisation</x:v>
+      </x:c>
+      <x:c r="B35" s="57" t="str">
+        <x:v>At least one complete up/down cycle or a clearly justified structural break</x:v>
+      </x:c>
+      <x:c r="C35" s="57" t="str">
+        <x:v>Normalize cycle earnings</x:v>
+      </x:c>
+      <x:c r="D35" s="57" t="str">
+        <x:v>Normalize DS segment only</x:v>
+      </x:c>
+      <x:c r="E35" s="57" t="str">
+        <x:v>Normalize NAND cycle only</x:v>
+      </x:c>
+      <x:c r="F35" s="62" t="str">
+        <x:v>Do not use peak/trough EPS PER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="24" hidden="0" customHeight="1">
+      <x:c r="A36" s="61" t="str">
+        <x:v>Valuation comparability</x:v>
+      </x:c>
+      <x:c r="B36" s="57" t="str">
+        <x:v>Same as-of date for price, FX, shares and net cash; disclose accounting adjustments</x:v>
+      </x:c>
+      <x:c r="C36" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="D36" s="57" t="str">
+        <x:v>Required for segment data</x:v>
+      </x:c>
+      <x:c r="E36" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="F36" s="62" t="str">
+        <x:v>Show a range or mark unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="63"/>
+      <x:c r="B37" s="64"/>
+      <x:c r="C37" s="64"/>
+      <x:c r="D37" s="64"/>
+      <x:c r="E37" s="64"/>
+      <x:c r="F37" s="65"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="83" t="str">
+        <x:v>PER bridge evidence policy</x:v>
+      </x:c>
+      <x:c r="B38" s="82"/>
+      <x:c r="C38" s="82"/>
+      <x:c r="D38" s="82"/>
+      <x:c r="E38" s="82"/>
+      <x:c r="F38" s="84"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="88" t="str">
+        <x:v>Factor</x:v>
+      </x:c>
+      <x:c r="B39" s="89" t="str">
+        <x:v>Observable input</x:v>
+      </x:c>
+      <x:c r="C39" s="89" t="str">
+        <x:v>Evidence that supports premium</x:v>
+      </x:c>
+      <x:c r="D39" s="89" t="str">
+        <x:v>Evidence that removes premium</x:v>
+      </x:c>
+      <x:c r="E39" s="89" t="str">
+        <x:v>Current workbook treatment</x:v>
+      </x:c>
+      <x:c r="F39" s="90" t="str">
+        <x:v>Review trigger</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="24" hidden="0" customHeight="1">
+      <x:c r="A40" s="61" t="str">
+        <x:v>HBM profit mix</x:v>
+      </x:c>
+      <x:c r="B40" s="57" t="str">
+        <x:v>HBM EBIT/revenue contribution by generation; public actuals separate from estimate</x:v>
+      </x:c>
+      <x:c r="C40" s="57" t="str">
+        <x:v>Sustained shipped volume, yield and cash contribution</x:v>
+      </x:c>
+      <x:c r="D40" s="57" t="str">
+        <x:v>Ramp delay, lower ASP, margin or yield</x:v>
+      </x:c>
+      <x:c r="E40" s="57" t="str">
+        <x:v>Base/Bull/Bear x inputs are analyst scenarios, not calibrated facts</x:v>
+      </x:c>
+      <x:c r="F40" s="62" t="str">
+        <x:v>Each earnings release / qualification update</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="24" hidden="0" customHeight="1">
+      <x:c r="A41" s="61" t="str">
+        <x:v>Growth duration</x:v>
+      </x:c>
+      <x:c r="B41" s="57" t="str">
+        <x:v>Customer qualification, platform adoption, next-generation transition</x:v>
+      </x:c>
+      <x:c r="C41" s="57" t="str">
+        <x:v>Multiple product generations with confirmed customer uptake</x:v>
+      </x:c>
+      <x:c r="D41" s="57" t="str">
+        <x:v>Single product/customer dependence or schedule slip</x:v>
+      </x:c>
+      <x:c r="E41" s="57" t="str">
+        <x:v>Narrative evidence first; no extra multiple without calibration</x:v>
+      </x:c>
+      <x:c r="F41" s="62" t="str">
+        <x:v>Every formal roadmap or earnings update</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="24" hidden="0" customHeight="1">
+      <x:c r="A42" s="61" t="str">
+        <x:v>Cash conversion</x:v>
+      </x:c>
+      <x:c r="B42" s="57" t="str">
+        <x:v>FCF/net income, CAPEX/revenue, inventory and receivable days</x:v>
+      </x:c>
+      <x:c r="C42" s="57" t="str">
+        <x:v>Profit growth converts to FCF after growth investment</x:v>
+      </x:c>
+      <x:c r="D42" s="57" t="str">
+        <x:v>Investment and working capital outgrow operating cash</x:v>
+      </x:c>
+      <x:c r="E42" s="57" t="str">
+        <x:v>Cross-check in DCF; avoid counting same benefit twice</x:v>
+      </x:c>
+      <x:c r="F42" s="62" t="str">
+        <x:v>Quarterly cash flow update</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="24" hidden="0" customHeight="1">
+      <x:c r="A43" s="61" t="str">
+        <x:v>Customer concentration</x:v>
+      </x:c>
+      <x:c r="B43" s="57" t="str">
+        <x:v>Disclosed customer mix or defensible proxy</x:v>
+      </x:c>
+      <x:c r="C43" s="57" t="str">
+        <x:v>Diversification and stable contracted demand</x:v>
+      </x:c>
+      <x:c r="D43" s="57" t="str">
+        <x:v>Order timing depends on few customers</x:v>
+      </x:c>
+      <x:c r="E43" s="57" t="str">
+        <x:v>Scenario haircut only; disclose if data unavailable</x:v>
+      </x:c>
+      <x:c r="F43" s="62" t="str">
+        <x:v>When customer/order disclosure changes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="24" hidden="0" customHeight="1">
+      <x:c r="A44" s="70" t="str">
+        <x:v>Cycle risk</x:v>
+      </x:c>
+      <x:c r="B44" s="71" t="str">
+        <x:v>ASP, inventory, bit supply and multi-year margins</x:v>
+      </x:c>
+      <x:c r="C44" s="71" t="str">
+        <x:v>Supply discipline and stable mid-cycle return on capital</x:v>
+      </x:c>
+      <x:c r="D44" s="71" t="str">
+        <x:v>Peak-cycle earnings or rapid supply response</x:v>
+      </x:c>
+      <x:c r="E44" s="71" t="str">
+        <x:v>Use cycle-normalised EPS; current x adjustments need backtest</x:v>
+      </x:c>
+      <x:c r="F44" s="72" t="str">
+        <x:v>Full-cycle refresh</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="24" hidden="0" customHeight="1">
+      <x:c r="A45" s="70" t="str">
+        <x:v>Multiple conversion</x:v>
+      </x:c>
+      <x:c r="B45" s="71" t="str">
+        <x:v>Historical peer-relative multiples across dates with same factor definitions</x:v>
+      </x:c>
+      <x:c r="C45" s="71" t="str">
+        <x:v>Observed repeatable relationship and adequate sample</x:v>
+      </x:c>
+      <x:c r="D45" s="71" t="str">
+        <x:v>No history, structural change or unstable coefficient</x:v>
+      </x:c>
+      <x:c r="E45" s="71" t="str">
+        <x:v>No calibrated premium claim until sample, period and error range are shown</x:v>
+      </x:c>
+      <x:c r="F45" s="72" t="str">
+        <x:v>At each annual model review</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
analysis: align Hynix RIM period and remove uncalibrated PER turns
</commit_message>
<xml_diff>
--- a/model/SK_hynix_equity_research_final.xlsx
+++ b/model/SK_hynix_equity_research_final.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R33c7b8cdcd2649a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="R2fd1dbaf8dab4638"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R28c35e5ef98c48a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HBM Build" sheetId="4" r:id="R066de7dfa4374f82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="5" r:id="R7c7762131c7e451c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" r:id="R1bc263dd514d47e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="7" r:id="Rb191f6435fc143d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="8" r:id="R536b6e46bb6b434d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="9" r:id="Rc50fd0b0ffc245af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R985789c6901848b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="Rdc731b14ddf342c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R8a7265b74b964501"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HBM Build" sheetId="4" r:id="R5632eb0b2d564288"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="5" r:id="R0d5be5fdfafe4c17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" r:id="R6ddf0898c0dc4834"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="7" r:id="R3d4d9981063e49d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="8" r:id="Rba9459651eec45d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="9" r:id="Rc04a2231785347a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -757,7 +757,7 @@
       </x:c>
       <x:c r="B10" s="29" t="n">
         <x:f>'Peer PER'!B27</x:f>
-        <x:v>1828571.428571429</x:v>
+        <x:v>1828571.4285714286</x:v>
       </x:c>
       <x:c r="C10" s="27" t="str">
         <x:v>Market cross-check</x:v>
@@ -775,7 +775,7 @@
       </x:c>
       <x:c r="B11" s="29" t="n">
         <x:f>'RIM'!B22</x:f>
-        <x:v>997094.5521517697</x:v>
+        <x:v>857492.1461555915</x:v>
       </x:c>
       <x:c r="C11" s="27" t="str">
         <x:v>Downside check</x:v>
@@ -3078,12 +3078,19 @@
       <x:c r="G2" s="6"/>
       <x:c r="H2" s="6"/>
     </x:row>
+    <x:row r="3">
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+    </x:row>
     <x:row r="4">
       <x:c r="A4" s="15" t="str">
         <x:v>Metric</x:v>
       </x:c>
       <x:c r="B4" s="15" t="str">
-        <x:v>2026E</x:v>
+        <x:v>2026H2</x:v>
       </x:c>
       <x:c r="C4" s="15" t="str">
         <x:v>2027E</x:v>
@@ -3103,19 +3110,23 @@
         <x:v>Opening equity</x:v>
       </x:c>
       <x:c r="B5" s="38" t="n">
-        <x:v>120516</x:v>
+        <x:v>169400</x:v>
       </x:c>
       <x:c r="C5" s="38" t="n">
-        <x:v>260000</x:v>
+        <x:f>B9</x:f>
+        <x:v>211198.625</x:v>
       </x:c>
       <x:c r="D5" s="38" t="n">
-        <x:v>372000</x:v>
+        <x:f>C9</x:f>
+        <x:v>323198.625</x:v>
       </x:c>
       <x:c r="E5" s="38" t="n">
-        <x:v>456000</x:v>
+        <x:f>D9</x:f>
+        <x:v>404448.625</x:v>
       </x:c>
       <x:c r="F5" s="38" t="n">
-        <x:v>522000</x:v>
+        <x:f>E9</x:f>
+        <x:v>461448.625</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -3123,7 +3134,8 @@
         <x:v>Net income</x:v>
       </x:c>
       <x:c r="B6" s="38" t="n">
-        <x:v>190000</x:v>
+        <x:f>'Forecast'!C8-'Actuals &amp; Sources'!D10-'Actuals &amp; Sources'!D13</x:f>
+        <x:v>55731.5</x:v>
       </x:c>
       <x:c r="C6" s="38" t="n">
         <x:v>160000</x:v>
@@ -3164,7 +3176,7 @@
       </x:c>
       <x:c r="B8" s="36" t="n">
         <x:f>B6*B7</x:f>
-        <x:v>47500</x:v>
+        <x:v>13932.875</x:v>
       </x:c>
       <x:c r="C8" s="36" t="n">
         <x:f>C6*C7</x:f>
@@ -3189,23 +3201,23 @@
       </x:c>
       <x:c r="B9" s="36" t="n">
         <x:f>B5+B6-B8</x:f>
-        <x:v>263016</x:v>
+        <x:v>211198.625</x:v>
       </x:c>
       <x:c r="C9" s="36" t="n">
         <x:f>C5+C6-C8</x:f>
-        <x:v>372000</x:v>
+        <x:v>323198.625</x:v>
       </x:c>
       <x:c r="D9" s="36" t="n">
         <x:f>D5+D6-D8</x:f>
-        <x:v>453250</x:v>
+        <x:v>404448.625</x:v>
       </x:c>
       <x:c r="E9" s="36" t="n">
         <x:f>E5+E6-E8</x:f>
-        <x:v>513000</x:v>
+        <x:v>461448.625</x:v>
       </x:c>
       <x:c r="F9" s="36" t="n">
         <x:f>F5+F6-F8</x:f>
-        <x:v>564900</x:v>
+        <x:v>504348.625</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -3213,24 +3225,24 @@
         <x:v>ROE</x:v>
       </x:c>
       <x:c r="B10" s="23" t="n">
-        <x:f>B6/B5</x:f>
-        <x:v>1.5765541504862426</x:v>
+        <x:f>B6/B5*2</x:f>
+        <x:v>0.657987012987013</x:v>
       </x:c>
       <x:c r="C10" s="23" t="n">
         <x:f>C6/C5</x:f>
-        <x:v>0.6153846153846154</x:v>
+        <x:v>0.7575806897417064</x:v>
       </x:c>
       <x:c r="D10" s="23" t="n">
         <x:f>D6/D5</x:f>
-        <x:v>0.33602150537634407</x:v>
+        <x:v>0.38675907114394437</x:v>
       </x:c>
       <x:c r="E10" s="23" t="n">
         <x:f>E6/E5</x:f>
-        <x:v>0.20833333333333334</x:v>
+        <x:v>0.23488768196455112</x:v>
       </x:c>
       <x:c r="F10" s="23" t="n">
         <x:f>F6/F5</x:f>
-        <x:v>0.14942528735632185</x:v>
+        <x:v>0.16903290154998296</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -3258,25 +3270,28 @@
         <x:v>Residual income</x:v>
       </x:c>
       <x:c r="B12" s="36" t="n">
-        <x:f>B6-B5*B11</x:f>
-        <x:v>177345.82</x:v>
+        <x:f>B6-B5*B11*0.5</x:f>
+        <x:v>46838</x:v>
       </x:c>
       <x:c r="C12" s="36" t="n">
         <x:f>C6-C5*C11</x:f>
-        <x:v>132700</x:v>
+        <x:v>137824.144375</x:v>
       </x:c>
       <x:c r="D12" s="36" t="n">
         <x:f>D6-D5*D11</x:f>
-        <x:v>85940</x:v>
+        <x:v>91064.144375</x:v>
       </x:c>
       <x:c r="E12" s="36" t="n">
         <x:f>E6-E5*E11</x:f>
-        <x:v>47120</x:v>
+        <x:v>52532.894375</x:v>
       </x:c>
       <x:c r="F12" s="36" t="n">
         <x:f>F6-F5*F11</x:f>
-        <x:v>23190</x:v>
-      </x:c>
+        <x:v>29547.894375000003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="B14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="15" t="str">
@@ -3288,9 +3303,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Starting equity (June 2026)</x:v>
+        <x:v>Starting equity (2026-06-30 reported)</x:v>
       </x:c>
       <x:c r="B16" s="40" t="n">
+        <x:f>B5</x:f>
         <x:v>169400</x:v>
       </x:c>
     </x:row>
@@ -3299,8 +3315,8 @@
         <x:v>PV residual income</x:v>
       </x:c>
       <x:c r="B17" s="40" t="n">
-        <x:f>B12/(1+B11)^1+C12/(1+C11)^2+D12/(1+D11)^3+E12/(1+E11)^4+F12/(1+F11)^5</x:f>
-        <x:v>378549.95829816605</x:v>
+        <x:f>B12/(1+B11)^0.5+C12/(1+C11)^1.5+D12/(1+D11)^2.5+E12/(1+E11)^3.5+F12/(1+F11)^4.5</x:f>
+        <x:v>290052.2853849265</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -3309,7 +3325,7 @@
       </x:c>
       <x:c r="B18" s="40" t="n">
         <x:f>F9*(B23-F11)/(F11-0.025)</x:f>
-        <x:v>247143.75000000017</x:v>
+        <x:v>220652.52343750015</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -3317,8 +3333,8 @@
         <x:v>PV terminal RI</x:v>
       </x:c>
       <x:c r="B19" s="40" t="n">
-        <x:f>B18/(1+F11)^5</x:f>
-        <x:v>150016.22820807275</x:v>
+        <x:f>B18/(1+F11)^4.5</x:f>
+        <x:v>140792.2169239876</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -3327,7 +3343,7 @@
       </x:c>
       <x:c r="B20" s="40" t="n">
         <x:f>B16+B17+B19</x:f>
-        <x:v>697966.1865062388</x:v>
+        <x:v>600244.5023089141</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -3344,7 +3360,7 @@
       </x:c>
       <x:c r="B22" s="40" t="n">
         <x:f>B20*1000/B21</x:f>
-        <x:v>997094.5521517697</x:v>
+        <x:v>857492.1461555915</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -3392,7 +3408,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Micron is the sole direct economics anchor. PER bridge values are analyst scenario inputs until historical calibration; see rows 30–45.</x:v>
+        <x:v>Micron is the sole direct economics anchor. Use direct 6x/8x/9x bear/base/bull anchors; qualitative factors do not become multiple turns without dated empirical calibration.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -3564,7 +3580,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="15" t="str">
-        <x:v>PER bridge</x:v>
+        <x:v>Micron anchor sensitivity; qualitative factors below are not translated into turns</x:v>
       </x:c>
       <x:c r="B14" s="15" t="str">
         <x:v>Base x</x:v>
@@ -3607,19 +3623,10 @@
       <x:c r="A16" s="27" t="str">
         <x:v>HBM profit mix</x:v>
       </x:c>
-      <x:c r="B16" s="48" t="n">
-        <x:v>0.8</x:v>
-      </x:c>
-      <x:c r="C16" s="48" t="n">
-        <x:v>1.2</x:v>
-      </x:c>
-      <x:c r="D16" s="48" t="n">
-        <x:v>0.2</x:v>
-      </x:c>
-      <x:c r="E16" s="49" t="n">
-        <x:f>IF(Summary!$B$4="Bull",C16,IF(Summary!$B$4="Bear",D16,B16))</x:f>
-        <x:v>0.8</x:v>
-      </x:c>
+      <x:c r="B16" s="48"/>
+      <x:c r="C16" s="48"/>
+      <x:c r="D16" s="48"/>
+      <x:c r="E16" s="49"/>
       <x:c r="F16" s="27" t="str">
         <x:v>Falls if HBM4 ramp/margin disappoints</x:v>
       </x:c>
@@ -3628,19 +3635,10 @@
       <x:c r="A17" s="27" t="str">
         <x:v>ROE quality</x:v>
       </x:c>
-      <x:c r="B17" s="48" t="n">
-        <x:v>0.4</x:v>
-      </x:c>
-      <x:c r="C17" s="48" t="n">
-        <x:v>0.6</x:v>
-      </x:c>
-      <x:c r="D17" s="48" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E17" s="49" t="n">
-        <x:f>IF(Summary!$B$4="Bull",C17,IF(Summary!$B$4="Bear",D17,B17))</x:f>
-        <x:v>0.4</x:v>
-      </x:c>
+      <x:c r="B17" s="48"/>
+      <x:c r="C17" s="48"/>
+      <x:c r="D17" s="48"/>
+      <x:c r="E17" s="49"/>
       <x:c r="F17" s="27" t="str">
         <x:v>Requires FCF-backed ROE</x:v>
       </x:c>
@@ -3649,19 +3647,10 @@
       <x:c r="A18" s="27" t="str">
         <x:v>Long-term supply visibility</x:v>
       </x:c>
-      <x:c r="B18" s="48" t="n">
-        <x:v>0.3</x:v>
-      </x:c>
-      <x:c r="C18" s="48" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="D18" s="48" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E18" s="49" t="n">
-        <x:f>IF(Summary!$B$4="Bull",C18,IF(Summary!$B$4="Bear",D18,B18))</x:f>
-        <x:v>0.3</x:v>
-      </x:c>
+      <x:c r="B18" s="48"/>
+      <x:c r="C18" s="48"/>
+      <x:c r="D18" s="48"/>
+      <x:c r="E18" s="49"/>
       <x:c r="F18" s="27" t="str">
         <x:v>Falls if LTA / qualification visibility fades</x:v>
       </x:c>
@@ -3670,19 +3659,10 @@
       <x:c r="A19" s="27" t="str">
         <x:v>Customer concentration</x:v>
       </x:c>
-      <x:c r="B19" s="48" t="n">
-        <x:v>-0.4</x:v>
-      </x:c>
-      <x:c r="C19" s="48" t="n">
-        <x:v>-0.2</x:v>
-      </x:c>
-      <x:c r="D19" s="48" t="n">
-        <x:v>-0.8</x:v>
-      </x:c>
-      <x:c r="E19" s="49" t="n">
-        <x:f>IF(Summary!$B$4="Bull",C19,IF(Summary!$B$4="Bear",D19,B19))</x:f>
-        <x:v>-0.4</x:v>
-      </x:c>
+      <x:c r="B19" s="48"/>
+      <x:c r="C19" s="48"/>
+      <x:c r="D19" s="48"/>
+      <x:c r="E19" s="49"/>
       <x:c r="F19" s="27" t="str">
         <x:v>Narrows with confirmed diversification</x:v>
       </x:c>
@@ -3691,19 +3671,10 @@
       <x:c r="A20" s="27" t="str">
         <x:v>CAPEX intensity</x:v>
       </x:c>
-      <x:c r="B20" s="48" t="n">
-        <x:v>-0.5</x:v>
-      </x:c>
-      <x:c r="C20" s="48" t="n">
-        <x:v>-0.3</x:v>
-      </x:c>
-      <x:c r="D20" s="48" t="n">
-        <x:v>-0.8</x:v>
-      </x:c>
-      <x:c r="E20" s="49" t="n">
-        <x:f>IF(Summary!$B$4="Bull",C20,IF(Summary!$B$4="Bear",D20,B20))</x:f>
-        <x:v>-0.5</x:v>
-      </x:c>
+      <x:c r="B20" s="48"/>
+      <x:c r="C20" s="48"/>
+      <x:c r="D20" s="48"/>
+      <x:c r="E20" s="49"/>
       <x:c r="F20" s="27" t="str">
         <x:v>Narrows only with FCF conversion</x:v>
       </x:c>
@@ -3712,19 +3683,10 @@
       <x:c r="A21" s="27" t="str">
         <x:v>Cycle volatility</x:v>
       </x:c>
-      <x:c r="B21" s="48" t="n">
-        <x:v>-0.6</x:v>
-      </x:c>
-      <x:c r="C21" s="48" t="n">
-        <x:v>-0.4</x:v>
-      </x:c>
-      <x:c r="D21" s="48" t="n">
-        <x:v>-1.2</x:v>
-      </x:c>
-      <x:c r="E21" s="49" t="n">
-        <x:f>IF(Summary!$B$4="Bull",C21,IF(Summary!$B$4="Bear",D21,B21))</x:f>
-        <x:v>-0.6</x:v>
-      </x:c>
+      <x:c r="B21" s="48"/>
+      <x:c r="C21" s="48"/>
+      <x:c r="D21" s="48"/>
+      <x:c r="E21" s="49"/>
       <x:c r="F21" s="27" t="str">
         <x:v>Narrows with supply discipline</x:v>
       </x:c>
@@ -3737,11 +3699,11 @@
       <x:c r="C22" s="27"/>
       <x:c r="D22" s="27"/>
       <x:c r="E22" s="49" t="n">
-        <x:f>SUM(E15:E21)</x:f>
-        <x:v>8.000000000000002</x:v>
+        <x:f>E15</x:f>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F22" s="27" t="str">
-        <x:v>Sum of anchor and adjustments</x:v>
+        <x:v>Selected direct peer anchor; no uncalibrated premium / discount arithmetic.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -3767,7 +3729,7 @@
       </x:c>
       <x:c r="B27" s="40" t="n">
         <x:f>B26*E22</x:f>
-        <x:v>1828571.428571429</x:v>
+        <x:v>1828571.4285714286</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -4203,7 +4165,7 @@
       </x:c>
       <x:c r="C10" s="37" t="n">
         <x:f>RIM!B22</x:f>
-        <x:v>997094.5521517697</x:v>
+        <x:v>857492.1461555915</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
         <x:v>PASS</x:v>

</xml_diff>

<commit_message>
analysis: align terminal residual income across company models
</commit_message>
<xml_diff>
--- a/model/SK_hynix_equity_research_final.xlsx
+++ b/model/SK_hynix_equity_research_final.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R985789c6901848b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="Rdc731b14ddf342c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R8a7265b74b964501"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HBM Build" sheetId="4" r:id="R5632eb0b2d564288"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="5" r:id="R0d5be5fdfafe4c17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" r:id="R6ddf0898c0dc4834"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="7" r:id="R3d4d9981063e49d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="8" r:id="Rba9459651eec45d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="9" r:id="Rc04a2231785347a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R970050ede3114ead"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="R4652664ec5e74f7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R5dae1bd94f4f43bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HBM Build" sheetId="4" r:id="R27bd6b232ae84205"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="5" r:id="Rf6943a6150a34b8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" r:id="R512ef881643e490c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="7" r:id="R9ab4c754f875474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="8" r:id="R9ce8356429b94871"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="9" r:id="R133d2b5adf644b0a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -775,7 +775,7 @@
       </x:c>
       <x:c r="B11" s="29" t="n">
         <x:f>'RIM'!B22</x:f>
-        <x:v>857492.1461555915</x:v>
+        <x:v>862520.4396171625</x:v>
       </x:c>
       <x:c r="C11" s="27" t="str">
         <x:v>Downside check</x:v>
@@ -3324,8 +3324,8 @@
         <x:v>Terminal RI value</x:v>
       </x:c>
       <x:c r="B18" s="40" t="n">
-        <x:f>F9*(B23-F11)/(F11-0.025)</x:f>
-        <x:v>220652.52343750015</x:v>
+        <x:f>F9*(B23-F11)*(1+0.025)/(F11-0.025)</x:f>
+        <x:v>226168.8365234376</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -3334,7 +3334,7 @@
       </x:c>
       <x:c r="B19" s="40" t="n">
         <x:f>B18/(1+F11)^4.5</x:f>
-        <x:v>140792.2169239876</x:v>
+        <x:v>144312.02234708727</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -3343,7 +3343,7 @@
       </x:c>
       <x:c r="B20" s="40" t="n">
         <x:f>B16+B17+B19</x:f>
-        <x:v>600244.5023089141</x:v>
+        <x:v>603764.3077320138</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -3360,7 +3360,7 @@
       </x:c>
       <x:c r="B22" s="40" t="n">
         <x:f>B20*1000/B21</x:f>
-        <x:v>857492.1461555915</x:v>
+        <x:v>862520.4396171625</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -4165,7 +4165,7 @@
       </x:c>
       <x:c r="C10" s="37" t="n">
         <x:f>RIM!B22</x:f>
-        <x:v>857492.1461555915</x:v>
+        <x:v>862520.4396171625</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
         <x:v>PASS</x:v>

</xml_diff>